<commit_message>
feat: Separate expenses and payroll into distinct modules
Refactor the expense management system to address client requirements for a fully independent "Gastos" module and a dedicated "Planillas" module.

- "Gastos" now focuses purely on general invoices and expenses, including invoice number, amount, date, and description, without associations to properties, employees, or categories.
- "Planillas" now manages labor costs (payroll entries) in its own `payroll_entries` table, retaining the necessary links to properties and employees.
- Enhance the "Gastos" page with new modals for adding, editing, and viewing expense details, alongside advanced filtering capabilities by date and amount ranges.
- Implement an Excel export feature for "Cobros", allowing users to download filtered charge data.
- Includes the `20260917000000_split_expenses_payroll.sql` migration to support the new database schema.
</commit_message>
<xml_diff>
--- a/public/plantilla-gastos.xlsx
+++ b/public/plantilla-gastos.xlsx
@@ -12,12 +12,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
-  <si>
-    <t>Propiedad</t>
-  </si>
-  <si>
-    <t>Categoria *</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+  <si>
+    <t>Numero de factura</t>
   </si>
   <si>
     <t>Monto *</t>
@@ -26,16 +23,13 @@
     <t>Fecha *</t>
   </si>
   <si>
-    <t>Empleado</t>
-  </si>
-  <si>
     <t>Descripcion</t>
   </si>
   <si>
     <t>Como llenar esta plantilla</t>
   </si>
   <si>
-    <t>Cada fila de la pestana "Gastos" es un gasto: pago de planilla a un empleado, compra de materiales, transporte, herramientas u otro gasto general. No hace falta llenar todas las columnas — solo Categoria, Monto y Fecha son obligatorias.</t>
+    <t>Cada fila de la pestana "Gastos" es una factura o gasto general. No esta ligado a propiedades, empleados ni categorias — solo Monto y Fecha son obligatorias.</t>
   </si>
   <si>
     <t>Columna</t>
@@ -44,10 +38,7 @@
     <t>Que va aqui</t>
   </si>
   <si>
-    <t>El nombre de la propiedad a la que pertenece el gasto. Se puede dejar en blanco si es un gasto general (no ligado a una propiedad especifica).</t>
-  </si>
-  <si>
-    <t>Una de: Materiales, Mano de obra, Transporte, Herramientas, Otro. Usa "Mano de obra" para pagos de planilla a empleados.</t>
+    <t>El numero de factura del gasto, si tiene uno. Se puede dejar en blanco.</t>
   </si>
   <si>
     <t>Monto en dolares, solo el numero (ej. 450 o 450.50, sin el signo $).</t>
@@ -56,10 +47,7 @@
     <t>Formato AAAA-MM-DD (ej. 2026-08-15).</t>
   </si>
   <si>
-    <t>Nombre del empleado al que se le pago. Si no existe, se crea. Solo tiene sentido cuando la categoria es "Mano de obra". Se puede dejar en blanco.</t>
-  </si>
-  <si>
-    <t>Cualquier detalle adicional del gasto (ej. "Pintura y brochas Home Depot", "Planilla quincenal 1-15 agosto"). Se puede dejar en blanco.</t>
+    <t>Cualquier detalle adicional del gasto (ej. "Pintura y brochas Home Depot", "Factura de gasolina agosto"). Se puede dejar en blanco.</t>
   </si>
 </sst>
 </file>
@@ -469,17 +457,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F300"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="34" customWidth="1"/>
+    <col min="2" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -492,321 +478,8 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="202" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="203" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="204" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="205" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="206" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="207" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="208" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="210" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="211" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="212" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="213" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="214" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="215" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="216" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="217" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="218" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="219" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="220" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="221" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="224" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="225" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="227" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="240" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="241" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="243" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="244" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="245" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="246" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="247" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="248" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="249" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="250" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="251" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="252" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="253" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="254" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="255" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="256" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="257" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="258" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="259" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="260" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="261" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="262" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="263" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="264" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="265" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="266" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="267" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="268" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="269" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="270" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="271" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="272" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="273" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="274" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="275" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="276" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="277" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="278" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="279" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="280" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="281" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="282" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="283" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="284" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="285" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="286" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="287" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="288" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="289" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="290" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="291" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="292" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="293" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="294" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="295" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="296" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="297" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="298" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="299" spans="2:2" x14ac:dyDescent="0.25"/>
-    <row r="300" spans="2:2" x14ac:dyDescent="0.25"/>
+    </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Categoria invalida" error="Elige una opcion de la lista." sqref="B10:B300">
-      <formula1>"Materiales,Mano de obra,Transporte,Herramientas,Otro"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Categoria invalida" error="Elige una opcion de la lista." sqref="B2:B300">
-      <formula1>"Materiales,Mano de obra,Transporte,Herramientas,Otro"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -814,7 +487,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -823,22 +496,22 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B1" s="2"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B2" s="3"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -846,7 +519,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -854,7 +527,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -862,7 +535,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -870,23 +543,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>